<commit_message>
Add loan management updates
</commit_message>
<xml_diff>
--- a/backend/data/loan_management.xlsx
+++ b/backend/data/loan_management.xlsx
@@ -12623,7 +12623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13424,6 +13424,90 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>LOG000019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>USR0001</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>LOGIN</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>AUTH</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>USR0001</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-08-15 12:45:13</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>User logged in</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>LOG000020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>USR0001</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>EMAIL</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>REPORTS</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-08-15 12:46:08</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Emailed report to vfffinance@gmail.com</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>